<commit_message>
Harden GPS navigator capability
</commit_message>
<xml_diff>
--- a/app/src/main/java/com/example/methodmesh/modules/gpstargetnavigator/docs/example_odk_gps_target_navigator.xlsx
+++ b/app/src/main/java/com/example/methodmesh/modules/gpstargetnavigator/docs/example_odk_gps_target_navigator.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I26"/>
+  <dimension ref="A1:I27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -645,7 +645,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>com.example.methodmesh.EXECUTE_METHOD(method_id='gps_target_navigator',input_target_name=${target_name_input},input_target_plus_code=${target_plus_code_input},input_target_latitude=${target_latitude_input},input_target_longitude=${target_longitude_input},input_arrival_radius_m=${arrival_radius_input},return_mode='flat')</t>
+          <t>com.example.methodmesh.EXECUTE_METHOD(method_id='gps_target_navigator',input_target_name=${target_name_input},input_target_plus_code=${target_plus_code_input},input_target_latitude=${target_latitude_input},input_target_longitude=${target_longitude_input},input_arrival_radius_m=${arrival_radius_input},input_payload_mode='FULL',return_mode='flat')</t>
         </is>
       </c>
     </row>
@@ -1004,27 +1004,49 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>navigation_summary</t>
+          <t>methodmesh_full_json</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Navigation: ${distance_m} m from ${target_name}; arrived=${arrived}</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>${methodmesh_status} != ''</t>
+          <t>MethodMesh metadata JSON</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>navigation_summary</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Navigation: ${distance_m} m from ${target_name}; arrived=${arrived}</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>${methodmesh_status} != ''</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
         <is>
           <t>end_group</t>
         </is>

</xml_diff>